<commit_message>
Polar column deconvolution notebook.
</commit_message>
<xml_diff>
--- a/Result/MZmine_Feature_List_37to44min_polar_column_RI.xlsx
+++ b/Result/MZmine_Feature_List_37to44min_polar_column_RI.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
   <si>
     <t xml:space="preserve">row ID</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">39_Leaves_5_polar.mzXML Peak height</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low ion match(&lt;5)</t>
   </si>
   <si>
     <t xml:space="preserve">Low match(&lt;700)</t>
@@ -659,7 +662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
         <v>5</v>
       </c>
@@ -671,6 +674,9 @@
       </c>
       <c r="D4" s="0" t="n">
         <v>2796.58758531037</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>48</v>
       </c>
       <c r="P4" s="0" t="n">
         <v>0</v>
@@ -786,7 +792,7 @@
         <v>2797.48131296718</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P5" s="0" t="n">
         <v>0</v>
@@ -1015,7 +1021,7 @@
         <v>2850.92579365079</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P7" s="0" t="n">
         <v>0</v>
@@ -1244,7 +1250,7 @@
         <v>2869.24409171076</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P9" s="0" t="n">
         <v>0</v>
@@ -1360,7 +1366,7 @@
         <v>2869.31216931217</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P10" s="0" t="n">
         <v>0</v>
@@ -1476,7 +1482,7 @@
         <v>2869.35626102293</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P11" s="0" t="n">
         <v>0</v>
@@ -1592,7 +1598,7 @@
         <v>2874.01895943563</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P12" s="0" t="n">
         <v>0</v>
@@ -1934,7 +1940,7 @@
         <v>2891.93121693122</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P15" s="0" t="n">
         <v>0</v>
@@ -2163,7 +2169,7 @@
         <v>2932.64037717602</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P17" s="0" t="n">
         <v>0</v>
@@ -2392,7 +2398,7 @@
         <v>2944.72234042553</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P19" s="0" t="n">
         <v>0</v>
@@ -3073,7 +3079,7 @@
         <v>2971.90556092843</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P25" s="0" t="n">
         <v>0</v>

</xml_diff>